<commit_message>
Classement : +18 secondes sur tous les temps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AvV6osJpsKJ5XRBArKiFJw
</commit_message>
<xml_diff>
--- a/classement.xlsx
+++ b/classement.xlsx
@@ -165,7 +165,7 @@
         </is>
       </c>
       <c r="G2" s="2">
-        <v>0.005787037037037037</v>
+        <v>0.0059953703703703705</v>
       </c>
       <c r="H2" s="3">
         <v>0.0</v>
@@ -210,7 +210,7 @@
         </is>
       </c>
       <c r="G3" s="2">
-        <v>0.005914351851851852</v>
+        <v>0.006122685185185185</v>
       </c>
       <c r="H3" s="3">
         <v>0.0</v>
@@ -255,7 +255,7 @@
         </is>
       </c>
       <c r="G4" s="2">
-        <v>0.005960648148148148</v>
+        <v>0.006168981481481482</v>
       </c>
       <c r="H4" s="3">
         <v>0.0</v>
@@ -300,7 +300,7 @@
         </is>
       </c>
       <c r="G5" s="2">
-        <v>0.006273148148148148</v>
+        <v>0.006481481481481481</v>
       </c>
       <c r="H5" s="3">
         <v>0.0</v>
@@ -345,7 +345,7 @@
         </is>
       </c>
       <c r="G6" s="2">
-        <v>0.006504629629629629</v>
+        <v>0.006712962962962963</v>
       </c>
       <c r="H6" s="3">
         <v>0.0</v>
@@ -390,7 +390,7 @@
         </is>
       </c>
       <c r="G7" s="2">
-        <v>0.006516203703703704</v>
+        <v>0.006724537037037037</v>
       </c>
       <c r="H7" s="3">
         <v>0.0</v>
@@ -435,7 +435,7 @@
         </is>
       </c>
       <c r="G8" s="2">
-        <v>0.006678240740740741</v>
+        <v>0.0068865740740740745</v>
       </c>
       <c r="H8" s="3">
         <v>0.0</v>
@@ -480,7 +480,7 @@
         </is>
       </c>
       <c r="G9" s="2">
-        <v>0.006701388888888889</v>
+        <v>0.0069097222222222225</v>
       </c>
       <c r="H9" s="3">
         <v>0.0</v>
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="G10" s="2">
-        <v>0.0067476851851851856</v>
+        <v>0.0069560185185185185</v>
       </c>
       <c r="H10" s="3">
         <v>0.0</v>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="G11" s="2">
-        <v>0.006782407407407407</v>
+        <v>0.006990740740740741</v>
       </c>
       <c r="H11" s="3">
         <v>0.0</v>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="G12" s="2">
-        <v>0.006875</v>
+        <v>0.007083333333333333</v>
       </c>
       <c r="H12" s="3">
         <v>0.0</v>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="G13" s="2">
-        <v>0.006967592592592593</v>
+        <v>0.007175925925925926</v>
       </c>
       <c r="H13" s="3">
         <v>0.0</v>
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="G14" s="2">
-        <v>0.007013888888888889</v>
+        <v>0.007222222222222222</v>
       </c>
       <c r="H14" s="3">
         <v>0.0</v>
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="G15" s="2">
-        <v>0.007048611111111111</v>
+        <v>0.007256944444444444</v>
       </c>
       <c r="H15" s="3">
         <v>0.0</v>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="G16" s="2">
-        <v>0.007094907407407407</v>
+        <v>0.00730324074074074</v>
       </c>
       <c r="H16" s="3">
         <v>0.0</v>
@@ -840,7 +840,7 @@
         </is>
       </c>
       <c r="G17" s="2">
-        <v>0.0071643518518518514</v>
+        <v>0.007372685185185185</v>
       </c>
       <c r="H17" s="3">
         <v>0.0</v>
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="G18" s="2">
-        <v>0.007222222222222222</v>
+        <v>0.007430555555555556</v>
       </c>
       <c r="H18" s="3">
         <v>0.0</v>
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="G19" s="2">
-        <v>0.007256944444444444</v>
+        <v>0.007465277777777778</v>
       </c>
       <c r="H19" s="3">
         <v>0.0</v>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="G20" s="2">
-        <v>0.007291666666666667</v>
+        <v>0.0075</v>
       </c>
       <c r="H20" s="3">
         <v>0.0</v>
@@ -1020,7 +1020,7 @@
         </is>
       </c>
       <c r="G21" s="2">
-        <v>0.007326388888888889</v>
+        <v>0.007534722222222222</v>
       </c>
       <c r="H21" s="3">
         <v>0.0</v>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="G22" s="2">
-        <v>0.007349537037037037</v>
+        <v>0.00755787037037037</v>
       </c>
       <c r="H22" s="3">
         <v>0.0</v>
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="G23" s="2">
-        <v>0.00738425925925926</v>
+        <v>0.007592592592592593</v>
       </c>
       <c r="H23" s="3">
         <v>0.0</v>
@@ -1155,7 +1155,7 @@
         </is>
       </c>
       <c r="G24" s="2">
-        <v>0.007442129629629629</v>
+        <v>0.007650462962962963</v>
       </c>
       <c r="H24" s="3">
         <v>0.0</v>
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="G25" s="2">
-        <v>0.007488425925925926</v>
+        <v>0.007696759259259259</v>
       </c>
       <c r="H25" s="3">
         <v>0.0</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="G26" s="2">
-        <v>0.0075</v>
+        <v>0.0077083333333333335</v>
       </c>
       <c r="H26" s="3">
         <v>0.0</v>
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="G27" s="2">
-        <v>0.0075</v>
+        <v>0.0077083333333333335</v>
       </c>
       <c r="H27" s="3">
         <v>0.0</v>
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="G28" s="2">
-        <v>0.007523148148148148</v>
+        <v>0.0077314814814814815</v>
       </c>
       <c r="H28" s="3">
         <v>0.0</v>
@@ -1380,7 +1380,7 @@
         </is>
       </c>
       <c r="G29" s="2">
-        <v>0.007592592592592593</v>
+        <v>0.0078009259259259256</v>
       </c>
       <c r="H29" s="3">
         <v>0.0</v>
@@ -1425,7 +1425,7 @@
         </is>
       </c>
       <c r="G30" s="2">
-        <v>0.00787037037037037</v>
+        <v>0.008078703703703704</v>
       </c>
       <c r="H30" s="3">
         <v>0.0</v>
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="G31" s="2">
-        <v>0.007893518518518518</v>
+        <v>0.008101851851851851</v>
       </c>
       <c r="H31" s="3">
         <v>0.0</v>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="G32" s="2">
-        <v>0.008043981481481482</v>
+        <v>0.008252314814814815</v>
       </c>
       <c r="H32" s="3">
         <v>0.0</v>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="G33" s="2">
-        <v>0.008078703703703704</v>
+        <v>0.008287037037037037</v>
       </c>
       <c r="H33" s="3">
         <v>0.0</v>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="G34" s="2">
-        <v>0.008113425925925927</v>
+        <v>0.00832175925925926</v>
       </c>
       <c r="H34" s="3">
         <v>0.0</v>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="G35" s="2">
-        <v>0.008125</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="H35" s="3">
         <v>0.0</v>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="G36" s="2">
-        <v>0.008148148148148147</v>
+        <v>0.008356481481481482</v>
       </c>
       <c r="H36" s="3">
         <v>0.0</v>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="G37" s="2">
-        <v>0.008194444444444445</v>
+        <v>0.008402777777777778</v>
       </c>
       <c r="H37" s="3">
         <v>0.0</v>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="G38" s="2">
-        <v>0.008287037037037037</v>
+        <v>0.00849537037037037</v>
       </c>
       <c r="H38" s="3">
         <v>0.0</v>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="G39" s="2">
-        <v>0.008356481481481482</v>
+        <v>0.008564814814814815</v>
       </c>
       <c r="H39" s="3">
         <v>0.0</v>
@@ -1870,7 +1870,7 @@
         </is>
       </c>
       <c r="G40" s="2">
-        <v>0.008368055555555556</v>
+        <v>0.008576388888888889</v>
       </c>
       <c r="H40" s="3">
         <v>0.0</v>
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="G41" s="2">
-        <v>0.008460648148148148</v>
+        <v>0.00866898148148148</v>
       </c>
       <c r="H41" s="3">
         <v>0.0</v>
@@ -1960,7 +1960,7 @@
         </is>
       </c>
       <c r="G42" s="2">
-        <v>0.008506944444444444</v>
+        <v>0.008715277777777778</v>
       </c>
       <c r="H42" s="3">
         <v>0.0</v>
@@ -2005,7 +2005,7 @@
         </is>
       </c>
       <c r="G43" s="2">
-        <v>0.008518518518518519</v>
+        <v>0.008726851851851852</v>
       </c>
       <c r="H43" s="3">
         <v>0.0</v>
@@ -2050,7 +2050,7 @@
         </is>
       </c>
       <c r="G44" s="2">
-        <v>0.008564814814814815</v>
+        <v>0.008773148148148148</v>
       </c>
       <c r="H44" s="3">
         <v>0.0</v>
@@ -2095,7 +2095,7 @@
         </is>
       </c>
       <c r="G45" s="2">
-        <v>0.008611111111111111</v>
+        <v>0.008819444444444444</v>
       </c>
       <c r="H45" s="3">
         <v>0.0</v>
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="G46" s="2">
-        <v>0.00869212962962963</v>
+        <v>0.008900462962962962</v>
       </c>
       <c r="H46" s="3">
         <v>0.0</v>
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="G47" s="2">
-        <v>0.008819444444444444</v>
+        <v>0.009027777777777777</v>
       </c>
       <c r="H47" s="3">
         <v>0.0</v>
@@ -2230,7 +2230,7 @@
         </is>
       </c>
       <c r="G48" s="2">
-        <v>0.00886574074074074</v>
+        <v>0.009074074074074075</v>
       </c>
       <c r="H48" s="3">
         <v>0.0</v>
@@ -2260,7 +2260,7 @@
         <v>1</v>
       </c>
       <c r="G49" s="2">
-        <v>0.008946759259259258</v>
+        <v>0.009155092592592593</v>
       </c>
       <c r="H49" s="3">
         <v>0.0</v>
@@ -2292,7 +2292,7 @@
         </is>
       </c>
       <c r="G50" s="2">
-        <v>0.008981481481481481</v>
+        <v>0.009189814814814816</v>
       </c>
       <c r="H50" s="3">
         <v>0.0</v>
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="G51" s="2">
-        <v>0.00900462962962963</v>
+        <v>0.009212962962962963</v>
       </c>
       <c r="H51" s="3">
         <v>0.0</v>
@@ -2382,7 +2382,7 @@
         </is>
       </c>
       <c r="G52" s="2">
-        <v>0.009108796296296297</v>
+        <v>0.00931712962962963</v>
       </c>
       <c r="H52" s="3">
         <v>0.0</v>
@@ -2427,7 +2427,7 @@
         </is>
       </c>
       <c r="G53" s="2">
-        <v>0.00912037037037037</v>
+        <v>0.009328703703703704</v>
       </c>
       <c r="H53" s="3">
         <v>0.0</v>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="G54" s="2">
-        <v>0.009131944444444444</v>
+        <v>0.009340277777777777</v>
       </c>
       <c r="H54" s="3">
         <v>0.0</v>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="G55" s="2">
-        <v>0.009131944444444444</v>
+        <v>0.009340277777777777</v>
       </c>
       <c r="H55" s="3">
         <v>0.0</v>
@@ -2547,7 +2547,7 @@
         <v>1</v>
       </c>
       <c r="G56" s="2">
-        <v>0.009143518518518518</v>
+        <v>0.009351851851851853</v>
       </c>
       <c r="H56" s="3">
         <v>0.0</v>
@@ -2579,7 +2579,7 @@
         </is>
       </c>
       <c r="G57" s="2">
-        <v>0.009155092592592593</v>
+        <v>0.009363425925925926</v>
       </c>
       <c r="H57" s="3">
         <v>0.0</v>
@@ -2624,7 +2624,7 @@
         </is>
       </c>
       <c r="G58" s="2">
-        <v>0.009467592592592593</v>
+        <v>0.009675925925925926</v>
       </c>
       <c r="H58" s="3">
         <v>0.0</v>
@@ -2669,7 +2669,7 @@
         </is>
       </c>
       <c r="G59" s="2">
-        <v>0.00949074074074074</v>
+        <v>0.009699074074074074</v>
       </c>
       <c r="H59" s="3">
         <v>0.0</v>
@@ -2714,7 +2714,7 @@
         </is>
       </c>
       <c r="G60" s="2">
-        <v>0.00949074074074074</v>
+        <v>0.009699074074074074</v>
       </c>
       <c r="H60" s="3">
         <v>0.0</v>
@@ -2759,7 +2759,7 @@
         </is>
       </c>
       <c r="G61" s="2">
-        <v>0.00949074074074074</v>
+        <v>0.009699074074074074</v>
       </c>
       <c r="H61" s="3">
         <v>0.0</v>
@@ -2804,7 +2804,7 @@
         </is>
       </c>
       <c r="G62" s="2">
-        <v>0.009502314814814814</v>
+        <v>0.009710648148148149</v>
       </c>
       <c r="H62" s="3">
         <v>0.0</v>
@@ -2849,7 +2849,7 @@
         </is>
       </c>
       <c r="G63" s="2">
-        <v>0.009502314814814814</v>
+        <v>0.009710648148148149</v>
       </c>
       <c r="H63" s="3">
         <v>0.0</v>
@@ -2894,7 +2894,7 @@
         </is>
       </c>
       <c r="G64" s="2">
-        <v>0.009502314814814814</v>
+        <v>0.009710648148148149</v>
       </c>
       <c r="H64" s="3">
         <v>0.0</v>
@@ -2939,7 +2939,7 @@
         </is>
       </c>
       <c r="G65" s="2">
-        <v>0.009502314814814814</v>
+        <v>0.009710648148148149</v>
       </c>
       <c r="H65" s="3">
         <v>0.0</v>
@@ -2979,7 +2979,7 @@
         </is>
       </c>
       <c r="G66" s="2">
-        <v>0.00951388888888889</v>
+        <v>0.009722222222222222</v>
       </c>
       <c r="H66" s="3">
         <v>0.0</v>
@@ -3024,7 +3024,7 @@
         </is>
       </c>
       <c r="G67" s="2">
-        <v>0.00951388888888889</v>
+        <v>0.009722222222222222</v>
       </c>
       <c r="H67" s="3">
         <v>0.0</v>
@@ -3069,7 +3069,7 @@
         </is>
       </c>
       <c r="G68" s="2">
-        <v>0.009525462962962963</v>
+        <v>0.009733796296296296</v>
       </c>
       <c r="H68" s="3">
         <v>0.0</v>
@@ -3114,7 +3114,7 @@
         </is>
       </c>
       <c r="G69" s="2">
-        <v>0.009525462962962963</v>
+        <v>0.009733796296296296</v>
       </c>
       <c r="H69" s="3">
         <v>0.0</v>
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="G70" s="2">
-        <v>0.009537037037037037</v>
+        <v>0.00974537037037037</v>
       </c>
       <c r="H70" s="3">
         <v>0.0</v>
@@ -3204,7 +3204,7 @@
         </is>
       </c>
       <c r="G71" s="2">
-        <v>0.009537037037037037</v>
+        <v>0.00974537037037037</v>
       </c>
       <c r="H71" s="3">
         <v>0.0</v>
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="G72" s="2">
-        <v>0.010162037037037037</v>
+        <v>0.01037037037037037</v>
       </c>
       <c r="H72" s="3">
         <v>0.0</v>
@@ -3294,7 +3294,7 @@
         </is>
       </c>
       <c r="G73" s="2">
-        <v>0.01017361111111111</v>
+        <v>0.010381944444444444</v>
       </c>
       <c r="H73" s="3">
         <v>0.0</v>
@@ -3339,7 +3339,7 @@
         </is>
       </c>
       <c r="G74" s="2">
-        <v>0.01019675925925926</v>
+        <v>0.010405092592592593</v>
       </c>
       <c r="H74" s="3">
         <v>0.0</v>
@@ -3384,7 +3384,7 @@
         </is>
       </c>
       <c r="G75" s="2">
-        <v>0.010300925925925925</v>
+        <v>0.01050925925925926</v>
       </c>
       <c r="H75" s="3">
         <v>0.0</v>
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="G76" s="2">
-        <v>0.010648148148148148</v>
+        <v>0.01085648148148148</v>
       </c>
       <c r="H76" s="3">
         <v>0.0</v>
@@ -3474,7 +3474,7 @@
         </is>
       </c>
       <c r="G77" s="2">
-        <v>0.010648148148148148</v>
+        <v>0.01085648148148148</v>
       </c>
       <c r="H77" s="3">
         <v>0.0</v>
@@ -3519,7 +3519,7 @@
         </is>
       </c>
       <c r="G78" s="2">
-        <v>0.010659722222222221</v>
+        <v>0.010868055555555556</v>
       </c>
       <c r="H78" s="3">
         <v>0.0</v>
@@ -3564,7 +3564,7 @@
         </is>
       </c>
       <c r="G79" s="2">
-        <v>0.010659722222222221</v>
+        <v>0.010868055555555556</v>
       </c>
       <c r="H79" s="3">
         <v>0.0</v>
@@ -3609,7 +3609,7 @@
         </is>
       </c>
       <c r="G80" s="2">
-        <v>0.010798611111111111</v>
+        <v>0.011006944444444444</v>
       </c>
       <c r="H80" s="3">
         <v>0.0</v>
@@ -3654,7 +3654,7 @@
         </is>
       </c>
       <c r="G81" s="2">
-        <v>0.011030092592592593</v>
+        <v>0.011238425925925926</v>
       </c>
       <c r="H81" s="3">
         <v>0.0</v>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="G82" s="2">
-        <v>0.011215277777777777</v>
+        <v>0.011423611111111112</v>
       </c>
       <c r="H82" s="3">
         <v>0.0</v>
@@ -3744,7 +3744,7 @@
         </is>
       </c>
       <c r="G83" s="2">
-        <v>0.011296296296296296</v>
+        <v>0.01150462962962963</v>
       </c>
       <c r="H83" s="3">
         <v>0.0</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="G84" s="2">
-        <v>0.01170138888888889</v>
+        <v>0.011909722222222223</v>
       </c>
       <c r="H84" s="3">
         <v>0.0</v>
@@ -3834,7 +3834,7 @@
         </is>
       </c>
       <c r="G85" s="2">
-        <v>0.011747685185185186</v>
+        <v>0.011956018518518519</v>
       </c>
       <c r="H85" s="3">
         <v>0.0</v>
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="G86" s="2">
-        <v>0.01175925925925926</v>
+        <v>0.011967592592592592</v>
       </c>
       <c r="H86" s="3">
         <v>0.0</v>
@@ -3924,7 +3924,7 @@
         </is>
       </c>
       <c r="G87" s="2">
-        <v>0.01175925925925926</v>
+        <v>0.011967592592592592</v>
       </c>
       <c r="H87" s="3">
         <v>0.0</v>
@@ -3969,7 +3969,7 @@
         </is>
       </c>
       <c r="G88" s="2">
-        <v>0.011770833333333333</v>
+        <v>0.011979166666666667</v>
       </c>
       <c r="H88" s="3">
         <v>0.0</v>
@@ -4014,7 +4014,7 @@
         </is>
       </c>
       <c r="G89" s="2">
-        <v>0.012650462962962962</v>
+        <v>0.012858796296296297</v>
       </c>
       <c r="H89" s="3">
         <v>0.0</v>
@@ -4059,7 +4059,7 @@
         </is>
       </c>
       <c r="G90" s="2">
-        <v>0.012650462962962962</v>
+        <v>0.012858796296296297</v>
       </c>
       <c r="H90" s="3">
         <v>0.0</v>
@@ -4104,7 +4104,7 @@
         </is>
       </c>
       <c r="G91" s="2">
-        <v>0.012650462962962962</v>
+        <v>0.012858796296296297</v>
       </c>
       <c r="H91" s="3">
         <v>0.0</v>
@@ -4149,7 +4149,7 @@
         </is>
       </c>
       <c r="G92" s="2">
-        <v>0.012650462962962962</v>
+        <v>0.012858796296296297</v>
       </c>
       <c r="H92" s="3">
         <v>0.0</v>
@@ -4194,7 +4194,7 @@
         </is>
       </c>
       <c r="G93" s="2">
-        <v>0.012662037037037038</v>
+        <v>0.01287037037037037</v>
       </c>
       <c r="H93" s="3">
         <v>0.0</v>
@@ -4239,7 +4239,7 @@
         </is>
       </c>
       <c r="G94" s="2">
-        <v>0.012662037037037038</v>
+        <v>0.01287037037037037</v>
       </c>
       <c r="H94" s="3">
         <v>0.0</v>
@@ -4284,7 +4284,7 @@
         </is>
       </c>
       <c r="G95" s="2">
-        <v>0.012673611111111111</v>
+        <v>0.012881944444444444</v>
       </c>
       <c r="H95" s="3">
         <v>0.0</v>
@@ -4329,7 +4329,7 @@
         </is>
       </c>
       <c r="G96" s="2">
-        <v>0.012685185185185185</v>
+        <v>0.012893518518518518</v>
       </c>
       <c r="H96" s="3">
         <v>0.0</v>
@@ -4364,7 +4364,7 @@
         </is>
       </c>
       <c r="G97" s="2">
-        <v>0.012685185185185185</v>
+        <v>0.012893518518518518</v>
       </c>
       <c r="H97" s="3">
         <v>0.0</v>
@@ -4409,7 +4409,7 @@
         </is>
       </c>
       <c r="G98" s="2">
-        <v>0.01269675925925926</v>
+        <v>0.012905092592592593</v>
       </c>
       <c r="H98" s="3">
         <v>0.0</v>
@@ -4454,7 +4454,7 @@
         </is>
       </c>
       <c r="G99" s="2">
-        <v>0.01269675925925926</v>
+        <v>0.012905092592592593</v>
       </c>
       <c r="H99" s="3">
         <v>0.0</v>
@@ -4499,7 +4499,7 @@
         </is>
       </c>
       <c r="G100" s="2">
-        <v>0.012708333333333334</v>
+        <v>0.012916666666666667</v>
       </c>
       <c r="H100" s="3">
         <v>0.0</v>
@@ -4544,7 +4544,7 @@
         </is>
       </c>
       <c r="G101" s="2">
-        <v>0.012708333333333334</v>
+        <v>0.012916666666666667</v>
       </c>
       <c r="H101" s="3">
         <v>0.0</v>
@@ -4589,7 +4589,7 @@
         </is>
       </c>
       <c r="G102" s="2">
-        <v>0.012719907407407407</v>
+        <v>0.01292824074074074</v>
       </c>
       <c r="H102" s="3">
         <v>0.0</v>
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="G103" s="2">
-        <v>0.013009259259259259</v>
+        <v>0.013217592592592593</v>
       </c>
       <c r="H103" s="3">
         <v>0.0</v>
@@ -4679,7 +4679,7 @@
         </is>
       </c>
       <c r="G104" s="2">
-        <v>0.013009259259259259</v>
+        <v>0.013217592592592593</v>
       </c>
       <c r="H104" s="3">
         <v>0.0</v>
@@ -4724,7 +4724,7 @@
         </is>
       </c>
       <c r="G105" s="2">
-        <v>0.013020833333333334</v>
+        <v>0.013229166666666667</v>
       </c>
       <c r="H105" s="3">
         <v>0.0</v>
@@ -4769,7 +4769,7 @@
         </is>
       </c>
       <c r="G106" s="2">
-        <v>0.01306712962962963</v>
+        <v>0.013275462962962963</v>
       </c>
       <c r="H106" s="3">
         <v>0.0</v>
@@ -4814,7 +4814,7 @@
         </is>
       </c>
       <c r="G107" s="2">
-        <v>0.013483796296296296</v>
+        <v>0.01369212962962963</v>
       </c>
       <c r="H107" s="3">
         <v>0.0</v>
@@ -4859,7 +4859,7 @@
         </is>
       </c>
       <c r="G108" s="2">
-        <v>0.013726851851851851</v>
+        <v>0.013935185185185186</v>
       </c>
       <c r="H108" s="3">
         <v>0.0</v>
@@ -4904,7 +4904,7 @@
         </is>
       </c>
       <c r="G109" s="2">
-        <v>0.014074074074074074</v>
+        <v>0.014282407407407407</v>
       </c>
       <c r="H109" s="3">
         <v>0.0</v>
@@ -4949,7 +4949,7 @@
         </is>
       </c>
       <c r="G110" s="2">
-        <v>0.014097222222222223</v>
+        <v>0.014305555555555556</v>
       </c>
       <c r="H110" s="3">
         <v>0.0</v>
@@ -4994,7 +4994,7 @@
         </is>
       </c>
       <c r="G111" s="2">
-        <v>0.014097222222222223</v>
+        <v>0.014305555555555556</v>
       </c>
       <c r="H111" s="3">
         <v>0.0</v>
@@ -5039,7 +5039,7 @@
         </is>
       </c>
       <c r="G112" s="2">
-        <v>0.014814814814814815</v>
+        <v>0.015023148148148148</v>
       </c>
       <c r="H112" s="3">
         <v>0.0</v>
@@ -5084,7 +5084,7 @@
         </is>
       </c>
       <c r="G113" s="2">
-        <v>0.014837962962962963</v>
+        <v>0.015046296296296295</v>
       </c>
       <c r="H113" s="3">
         <v>0.0</v>

</xml_diff>

<commit_message>
Classement : ajout d'un troisième onglet « Classement 3 » (41 lignes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FwET4s16MrKdCfDDRhZPhg
</commit_message>
<xml_diff>
--- a/classement.xlsx
+++ b/classement.xlsx
@@ -4,10 +4,12 @@
   <sheets>
     <sheet name="Classement" sheetId="1" r:id="rId1"/>
     <sheet name="Classement 2" sheetId="2" r:id="rId3"/>
+    <sheet name="Classement 3" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Classement!$A$1:$O$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Classement 2'!$A$1:$O$216</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Classement 3'!$A$1:$O$42</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -14606,4 +14608,1852 @@
   </sheetData>
   <autoFilter ref="A1:O216"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="7" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="3" customWidth="1"/>
+    <col min="7" max="7" width="9" customWidth="1"/>
+    <col min="8" max="8" width="9" customWidth="1"/>
+    <col min="9" max="9" width="3" customWidth="1"/>
+    <col min="10" max="10" width="3" customWidth="1"/>
+    <col min="11" max="11" width="7" customWidth="1"/>
+    <col min="12" max="12" width="8" customWidth="1"/>
+    <col min="13" max="13" width="3" customWidth="1"/>
+    <col min="14" max="14" width="7" customWidth="1"/>
+    <col min="15" max="15" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>Clt</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t>Tours</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>Prénom</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t>Classe</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr" s="1">
+        <is>
+          <t>Temps</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr" s="1">
+        <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr" s="1">
+        <is>
+          <t>Rang</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr" s="1">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr" s="1">
+        <is>
+          <t>Sexe</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr" s="1">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DONNEZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nino</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G2" s="2">
+        <v>0.007013888888888889</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K2" s="4">
+        <v>2</v>
+      </c>
+      <c r="L2" s="4">
+        <v>8</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Minime 2 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DEBUIRE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Victor</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G3" s="2">
+        <v>0.009965277777777778</v>
+      </c>
+      <c r="H3" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K3" s="4">
+        <v>5</v>
+      </c>
+      <c r="L3" s="4">
+        <v>8</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Cadet M</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ROCROY</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ethan</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G4" s="2">
+        <v>0.010011574074074074</v>
+      </c>
+      <c r="H4" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K4" s="4">
+        <v>7</v>
+      </c>
+      <c r="L4" s="4">
+        <v>8</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Minime 2 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>DEROEUX</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Aaron</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G5" s="2">
+        <v>0.010034722222222223</v>
+      </c>
+      <c r="H5" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K5" s="4">
+        <v>10</v>
+      </c>
+      <c r="L5" s="4">
+        <v>8</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>WYCKAERT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Lucas</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G6" s="2">
+        <v>0.010046296296296296</v>
+      </c>
+      <c r="H6" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K6" s="4">
+        <v>12</v>
+      </c>
+      <c r="L6" s="4">
+        <v>8</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ROCHE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Timothé</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G7" s="2">
+        <v>0.010046296296296296</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K7" s="4">
+        <v>15</v>
+      </c>
+      <c r="L7" s="4">
+        <v>8</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>HACCART</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Lucas</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G8" s="2">
+        <v>0.010046296296296296</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K8" s="4">
+        <v>17</v>
+      </c>
+      <c r="L8" s="4">
+        <v>7</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Cadet M</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BOULET</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Léo</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G9" s="2">
+        <v>0.010046296296296296</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K9" s="4">
+        <v>20</v>
+      </c>
+      <c r="L9" s="4">
+        <v>7</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Minime 2 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CARPENTIER</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Antonin</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G10" s="2">
+        <v>0.01005787037037037</v>
+      </c>
+      <c r="H10" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K10" s="4">
+        <v>22</v>
+      </c>
+      <c r="L10" s="4">
+        <v>7</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Cadet M</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4">
+        <v>1</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>LEFEVRE COUPE</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Elora</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G11" s="2">
+        <v>0.01005787037037037</v>
+      </c>
+      <c r="H11" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K11" s="4">
+        <v>24</v>
+      </c>
+      <c r="L11" s="4">
+        <v>7</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Cadet F</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4">
+        <v>1</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DEVAUCHELLE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Tyméo</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G12" s="2">
+        <v>0.010081018518518519</v>
+      </c>
+      <c r="H12" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K12" s="4">
+        <v>27</v>
+      </c>
+      <c r="L12" s="4">
+        <v>7</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4">
+        <v>1</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DESFRANCOIS</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Lucas</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G13" s="2">
+        <v>0.010092592592592592</v>
+      </c>
+      <c r="H13" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K13" s="4">
+        <v>29</v>
+      </c>
+      <c r="L13" s="4">
+        <v>7</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LAMOUR</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Hugo</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G14" s="2">
+        <v>0.010208333333333333</v>
+      </c>
+      <c r="H14" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K14" s="4">
+        <v>32</v>
+      </c>
+      <c r="L14" s="4">
+        <v>6</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ROUGEGREZ</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Mael</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G15" s="2">
+        <v>0.01056712962962963</v>
+      </c>
+      <c r="H15" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K15" s="4">
+        <v>34</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4">
+        <v>1</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>GELE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Yanis</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G16" s="2">
+        <v>0.010578703703703703</v>
+      </c>
+      <c r="H16" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K16" s="4">
+        <v>37</v>
+      </c>
+      <c r="L16" s="4">
+        <v>6</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Minime 2 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PROBIN</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tristan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G17" s="2">
+        <v>0.010590277777777778</v>
+      </c>
+      <c r="H17" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K17" s="4">
+        <v>39</v>
+      </c>
+      <c r="L17" s="4">
+        <v>6</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Minime 2 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4">
+        <v>1</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>VALCKE</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Aloïs</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G18" s="2">
+        <v>0.010694444444444444</v>
+      </c>
+      <c r="H18" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K18" s="4">
+        <v>41</v>
+      </c>
+      <c r="L18" s="4">
+        <v>5</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4">
+        <v>1</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>LASSALLE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Mathys</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G19" s="2">
+        <v>0.010717592592592593</v>
+      </c>
+      <c r="H19" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K19" s="4">
+        <v>44</v>
+      </c>
+      <c r="L19" s="4">
+        <v>5</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4">
+        <v>1</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>HELLEBOID</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Roméo</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G20" s="2">
+        <v>0.01074074074074074</v>
+      </c>
+      <c r="H20" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K20" s="4">
+        <v>46</v>
+      </c>
+      <c r="L20" s="4">
+        <v>5</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4">
+        <v>1</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>DESPICHT</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Pauline</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G21" s="2">
+        <v>0.010775462962962962</v>
+      </c>
+      <c r="H21" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K21" s="4">
+        <v>49</v>
+      </c>
+      <c r="L21" s="4">
+        <v>5</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Cadet F</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CAZENAVE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Camille</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G22" s="2">
+        <v>0.011087962962962963</v>
+      </c>
+      <c r="H22" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K22" s="4">
+        <v>51</v>
+      </c>
+      <c r="L22" s="4">
+        <v>4</v>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Minime 1 F</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4">
+        <v>22</v>
+      </c>
+      <c r="B23" s="4">
+        <v>1</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>LEGROS</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Gabriel</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G23" s="2">
+        <v>0.01136574074074074</v>
+      </c>
+      <c r="H23" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K23" s="4">
+        <v>54</v>
+      </c>
+      <c r="L23" s="4">
+        <v>4</v>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Minime 2 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4">
+        <v>23</v>
+      </c>
+      <c r="B24" s="4">
+        <v>1</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>DELMOTTE</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Timéo</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G24" s="2">
+        <v>0.011817129629629629</v>
+      </c>
+      <c r="H24" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K24" s="4">
+        <v>56</v>
+      </c>
+      <c r="L24" s="4">
+        <v>4</v>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4">
+        <v>1</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>LAGNEAU</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Louis</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G25" s="2">
+        <v>0.011967592592592592</v>
+      </c>
+      <c r="H25" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K25" s="4">
+        <v>59</v>
+      </c>
+      <c r="L25" s="4">
+        <v>4</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Minime 2 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4">
+        <v>1</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0.012291666666666666</v>
+      </c>
+      <c r="H26" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K26" s="4">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4">
+        <v>1</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>JOSEFOWICZ</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Louis</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G27" s="2">
+        <v>0.012303240740740741</v>
+      </c>
+      <c r="H27" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K27" s="4">
+        <v>63</v>
+      </c>
+      <c r="L27" s="4">
+        <v>3</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Minime 2 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4">
+        <v>27</v>
+      </c>
+      <c r="B28" s="4">
+        <v>1</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>DUCHENE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Jules</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G28" s="2">
+        <v>0.012476851851851852</v>
+      </c>
+      <c r="H28" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K28" s="4">
+        <v>66</v>
+      </c>
+      <c r="L28" s="4">
+        <v>3</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4">
+        <v>1</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Dufour</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Marie</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G29" s="2">
+        <v>0.012835648148148148</v>
+      </c>
+      <c r="H29" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K29" s="4">
+        <v>68</v>
+      </c>
+      <c r="L29" s="4">
+        <v>3</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Minime 1 F</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4">
+        <v>1</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Mychaux</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Chstyele</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G30" s="2">
+        <v>0.01287037037037037</v>
+      </c>
+      <c r="H30" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K30" s="4">
+        <v>71</v>
+      </c>
+      <c r="L30" s="4">
+        <v>3</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Minime 1 F</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4">
+        <v>1</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>DUQUENNE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Arthur</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G31" s="2">
+        <v>0.012905092592592593</v>
+      </c>
+      <c r="H31" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K31" s="4">
+        <v>73</v>
+      </c>
+      <c r="L31" s="4">
+        <v>3</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Minime M</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4">
+        <v>31</v>
+      </c>
+      <c r="B32" s="4">
+        <v>1</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>DUFRESNE</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Louis</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G32" s="2">
+        <v>0.013113425925925926</v>
+      </c>
+      <c r="H32" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K32" s="4">
+        <v>76</v>
+      </c>
+      <c r="L32" s="4">
+        <v>2</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4">
+        <v>32</v>
+      </c>
+      <c r="B33" s="4">
+        <v>1</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>DUPONT</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Alban</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G33" s="2">
+        <v>0.013657407407407408</v>
+      </c>
+      <c r="H33" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K33" s="4">
+        <v>78</v>
+      </c>
+      <c r="L33" s="4">
+        <v>2</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4">
+        <v>33</v>
+      </c>
+      <c r="B34" s="4">
+        <v>1</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PIETRZAK VERET</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Stefan</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G34" s="2">
+        <v>0.013703703703703704</v>
+      </c>
+      <c r="H34" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K34" s="4">
+        <v>80</v>
+      </c>
+      <c r="L34" s="4">
+        <v>2</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4">
+        <v>34</v>
+      </c>
+      <c r="B35" s="4">
+        <v>1</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MEILLIEZ</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Antoine</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G35" s="2">
+        <v>0.014189814814814815</v>
+      </c>
+      <c r="H35" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K35" s="4">
+        <v>83</v>
+      </c>
+      <c r="L35" s="4">
+        <v>2</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4">
+        <v>35</v>
+      </c>
+      <c r="B36" s="4">
+        <v>1</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>HENRY</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Nathanaël</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G36" s="2">
+        <v>0.014293981481481482</v>
+      </c>
+      <c r="H36" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K36" s="4">
+        <v>85</v>
+      </c>
+      <c r="L36" s="4">
+        <v>2</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4">
+        <v>36</v>
+      </c>
+      <c r="B37" s="4">
+        <v>1</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="G37" s="2">
+        <v>0.014351851851851852</v>
+      </c>
+      <c r="H37" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K37" s="4">
+        <v>88</v>
+      </c>
+      <c r="L37" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4">
+        <v>37</v>
+      </c>
+      <c r="B38" s="4">
+        <v>1</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>DELMOTTE</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Margaux</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TROISIEME</t>
+        </is>
+      </c>
+      <c r="G38" s="2">
+        <v>0.014548611111111111</v>
+      </c>
+      <c r="H38" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K38" s="4">
+        <v>90</v>
+      </c>
+      <c r="L38" s="4">
+        <v>1</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Minime 2 F</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4">
+        <v>38</v>
+      </c>
+      <c r="B39" s="4">
+        <v>1</v>
+      </c>
+      <c r="G39" s="2">
+        <v>0.016215277777777776</v>
+      </c>
+      <c r="H39" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K39" s="4">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4">
+        <v>39</v>
+      </c>
+      <c r="B40" s="4">
+        <v>1</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CARON</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Alvin</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G40" s="2">
+        <v>0.01625</v>
+      </c>
+      <c r="H40" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K40" s="4">
+        <v>95</v>
+      </c>
+      <c r="L40" s="4">
+        <v>1</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4">
+        <v>40</v>
+      </c>
+      <c r="B41" s="4">
+        <v>1</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>DELATTRE</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Lucenzo</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G41" s="2">
+        <v>0.016354166666666666</v>
+      </c>
+      <c r="H41" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K41" s="4">
+        <v>98</v>
+      </c>
+      <c r="L41" s="4">
+        <v>1</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4">
+        <v>41</v>
+      </c>
+      <c r="B42" s="4">
+        <v>1</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MARATIER-FLAHAUT</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Manoey</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>QUATRIEME</t>
+        </is>
+      </c>
+      <c r="G42" s="2">
+        <v>0.017025462962962964</v>
+      </c>
+      <c r="H42" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="K42" s="4">
+        <v>100</v>
+      </c>
+      <c r="L42" s="4">
+        <v>0</v>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Minime 1 M</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O42"/>
+</worksheet>
 </file>
</xml_diff>